<commit_message>
Refresh report-round-trip E2E artifacts
Byproducts of running scripts/e2eReportRoundTrip.mjs to verify the Import UI
is still reachable under VITE_E2E after hiding it in production (17/17
passed). Screenshots and the downloaded workbook now reflect the current
build; no code or expectations changed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T4LurPsVU5WNa1i8str9pz
</commit_message>
<xml_diff>
--- a/e2e-screenshots/report-round-trip/downloaded-inventory-report.xlsx
+++ b/e2e-screenshots/report-round-trip/downloaded-inventory-report.xlsx
@@ -1112,7 +1112,7 @@
         <v>21</v>
       </c>
       <c r="L2">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -1150,7 +1150,7 @@
         <v>21</v>
       </c>
       <c r="L3">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -1188,7 +1188,7 @@
         <v>21</v>
       </c>
       <c r="L4">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -1226,7 +1226,7 @@
         <v>21</v>
       </c>
       <c r="L5">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -1264,7 +1264,7 @@
         <v>21</v>
       </c>
       <c r="L6">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
@@ -1302,7 +1302,7 @@
         <v>21</v>
       </c>
       <c r="L7">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
@@ -1340,7 +1340,7 @@
         <v>21</v>
       </c>
       <c r="L8">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
@@ -1378,7 +1378,7 @@
         <v>21</v>
       </c>
       <c r="L9">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
@@ -1416,7 +1416,7 @@
         <v>21</v>
       </c>
       <c r="L10">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
@@ -1454,7 +1454,7 @@
         <v>21</v>
       </c>
       <c r="L11">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
@@ -1492,7 +1492,7 @@
         <v>21</v>
       </c>
       <c r="L12">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
@@ -1530,7 +1530,7 @@
         <v>21</v>
       </c>
       <c r="L13">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
@@ -1568,7 +1568,7 @@
         <v>21</v>
       </c>
       <c r="L14">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
@@ -1606,7 +1606,7 @@
         <v>21</v>
       </c>
       <c r="L15">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
@@ -1644,7 +1644,7 @@
         <v>21</v>
       </c>
       <c r="L16">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
@@ -1682,7 +1682,7 @@
         <v>21</v>
       </c>
       <c r="L17">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
@@ -1720,7 +1720,7 @@
         <v>21</v>
       </c>
       <c r="L18">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
@@ -1758,7 +1758,7 @@
         <v>21</v>
       </c>
       <c r="L19">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
@@ -1796,7 +1796,7 @@
         <v>21</v>
       </c>
       <c r="L20">
-        <v>17</v>
+        <v>22</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
@@ -1834,7 +1834,7 @@
         <v>21</v>
       </c>
       <c r="L21">
-        <v>17</v>
+        <v>22</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
@@ -1872,7 +1872,7 @@
         <v>21</v>
       </c>
       <c r="L22">
-        <v>18</v>
+        <v>23</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
@@ -1910,7 +1910,7 @@
         <v>21</v>
       </c>
       <c r="L23">
-        <v>18</v>
+        <v>23</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
@@ -1948,7 +1948,7 @@
         <v>21</v>
       </c>
       <c r="L24">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
@@ -1986,7 +1986,7 @@
         <v>21</v>
       </c>
       <c r="L25">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
@@ -2024,7 +2024,7 @@
         <v>21</v>
       </c>
       <c r="L26">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
@@ -2062,7 +2062,7 @@
         <v>21</v>
       </c>
       <c r="L27">
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
@@ -2100,7 +2100,7 @@
         <v>21</v>
       </c>
       <c r="L28">
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
@@ -2138,7 +2138,7 @@
         <v>21</v>
       </c>
       <c r="L29">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
@@ -2176,7 +2176,7 @@
         <v>21</v>
       </c>
       <c r="L30">
-        <v>23</v>
+        <v>28</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
@@ -2214,7 +2214,7 @@
         <v>21</v>
       </c>
       <c r="L31">
-        <v>23</v>
+        <v>28</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
@@ -2252,7 +2252,7 @@
         <v>21</v>
       </c>
       <c r="L32">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
@@ -2290,7 +2290,7 @@
         <v>21</v>
       </c>
       <c r="L33">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.25">
@@ -2328,7 +2328,7 @@
         <v>21</v>
       </c>
       <c r="L34">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.25">
@@ -2366,7 +2366,7 @@
         <v>21</v>
       </c>
       <c r="L35">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.25">
@@ -2404,7 +2404,7 @@
         <v>21</v>
       </c>
       <c r="L36">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.25">
@@ -2442,7 +2442,7 @@
         <v>21</v>
       </c>
       <c r="L37">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.25">
@@ -2480,7 +2480,7 @@
         <v>21</v>
       </c>
       <c r="L38">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.25">
@@ -2518,7 +2518,7 @@
         <v>21</v>
       </c>
       <c r="L39">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.25">
@@ -2556,7 +2556,7 @@
         <v>21</v>
       </c>
       <c r="L40">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.25">
@@ -2594,7 +2594,7 @@
         <v>21</v>
       </c>
       <c r="L41">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.25">
@@ -2632,7 +2632,7 @@
         <v>21</v>
       </c>
       <c r="L42">
-        <v>29</v>
+        <v>34</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.25">
@@ -2670,7 +2670,7 @@
         <v>21</v>
       </c>
       <c r="L43">
-        <v>29</v>
+        <v>34</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
@@ -2708,7 +2708,7 @@
         <v>21</v>
       </c>
       <c r="L44">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.25">
@@ -2746,7 +2746,7 @@
         <v>21</v>
       </c>
       <c r="L45">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.25">
@@ -2784,7 +2784,7 @@
         <v>21</v>
       </c>
       <c r="L46">
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.25">
@@ -2822,7 +2822,7 @@
         <v>21</v>
       </c>
       <c r="L47">
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.25">
@@ -2860,7 +2860,7 @@
         <v>21</v>
       </c>
       <c r="L48">
-        <v>32</v>
+        <v>37</v>
       </c>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.25">
@@ -2898,7 +2898,7 @@
         <v>21</v>
       </c>
       <c r="L49">
-        <v>33</v>
+        <v>38</v>
       </c>
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.25">
@@ -2936,7 +2936,7 @@
         <v>21</v>
       </c>
       <c r="L50">
-        <v>33</v>
+        <v>38</v>
       </c>
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.25">
@@ -2974,7 +2974,7 @@
         <v>21</v>
       </c>
       <c r="L51">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.25">
@@ -3012,7 +3012,7 @@
         <v>21</v>
       </c>
       <c r="L52">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.25">
@@ -3050,7 +3050,7 @@
         <v>21</v>
       </c>
       <c r="L53">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.25">
@@ -3088,7 +3088,7 @@
         <v>21</v>
       </c>
       <c r="L54">
-        <v>36</v>
+        <v>41</v>
       </c>
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.25">
@@ -3126,7 +3126,7 @@
         <v>21</v>
       </c>
       <c r="L55">
-        <v>36</v>
+        <v>41</v>
       </c>
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.25">
@@ -3164,7 +3164,7 @@
         <v>21</v>
       </c>
       <c r="L56">
-        <v>37</v>
+        <v>42</v>
       </c>
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.25">
@@ -3202,7 +3202,7 @@
         <v>21</v>
       </c>
       <c r="L57">
-        <v>37</v>
+        <v>42</v>
       </c>
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.25">
@@ -3240,7 +3240,7 @@
         <v>21</v>
       </c>
       <c r="L58">
-        <v>37</v>
+        <v>42</v>
       </c>
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.25">
@@ -3278,7 +3278,7 @@
         <v>21</v>
       </c>
       <c r="L59">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.25">
@@ -3316,7 +3316,7 @@
         <v>21</v>
       </c>
       <c r="L60">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.25">
@@ -3354,7 +3354,7 @@
         <v>21</v>
       </c>
       <c r="L61">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.25">
@@ -3392,7 +3392,7 @@
         <v>21</v>
       </c>
       <c r="L62">
-        <v>39</v>
+        <v>44</v>
       </c>
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.25">
@@ -3430,7 +3430,7 @@
         <v>21</v>
       </c>
       <c r="L63">
-        <v>39</v>
+        <v>44</v>
       </c>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.25">
@@ -3468,7 +3468,7 @@
         <v>21</v>
       </c>
       <c r="L64">
-        <v>39</v>
+        <v>44</v>
       </c>
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.25">
@@ -3506,7 +3506,7 @@
         <v>21</v>
       </c>
       <c r="L65">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.25">
@@ -3544,7 +3544,7 @@
         <v>21</v>
       </c>
       <c r="L66">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.25">
@@ -3582,7 +3582,7 @@
         <v>21</v>
       </c>
       <c r="L67">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="68" spans="1:12" x14ac:dyDescent="0.25">
@@ -3620,7 +3620,7 @@
         <v>21</v>
       </c>
       <c r="L68">
-        <v>41</v>
+        <v>46</v>
       </c>
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.25">
@@ -3658,7 +3658,7 @@
         <v>21</v>
       </c>
       <c r="L69">
-        <v>41</v>
+        <v>46</v>
       </c>
     </row>
     <row r="70" spans="1:12" x14ac:dyDescent="0.25">
@@ -3696,7 +3696,7 @@
         <v>21</v>
       </c>
       <c r="L70">
-        <v>41</v>
+        <v>46</v>
       </c>
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.25">
@@ -3734,7 +3734,7 @@
         <v>21</v>
       </c>
       <c r="L71">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>21</v>
       </c>
       <c r="L72">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.25">
@@ -3810,7 +3810,7 @@
         <v>21</v>
       </c>
       <c r="L73">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.25">
@@ -3848,7 +3848,7 @@
         <v>21</v>
       </c>
       <c r="L74">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.25">
@@ -3886,7 +3886,7 @@
         <v>21</v>
       </c>
       <c r="L75">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="76" spans="1:12" x14ac:dyDescent="0.25">
@@ -3924,7 +3924,7 @@
         <v>21</v>
       </c>
       <c r="L76">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.25">
@@ -3962,7 +3962,7 @@
         <v>21</v>
       </c>
       <c r="L77">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="78" spans="1:12" x14ac:dyDescent="0.25">
@@ -4000,7 +4000,7 @@
         <v>21</v>
       </c>
       <c r="L78">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="79" spans="1:12" x14ac:dyDescent="0.25">
@@ -4038,7 +4038,7 @@
         <v>21</v>
       </c>
       <c r="L79">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="80" spans="1:12" x14ac:dyDescent="0.25">
@@ -4076,7 +4076,7 @@
         <v>21</v>
       </c>
       <c r="L80">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.25">
@@ -4114,7 +4114,7 @@
         <v>21</v>
       </c>
       <c r="L81">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="82" spans="1:12" x14ac:dyDescent="0.25">
@@ -4152,7 +4152,7 @@
         <v>21</v>
       </c>
       <c r="L82">
-        <v>46</v>
+        <v>51</v>
       </c>
     </row>
     <row r="83" spans="1:12" x14ac:dyDescent="0.25">
@@ -4190,7 +4190,7 @@
         <v>21</v>
       </c>
       <c r="L83">
-        <v>46</v>
+        <v>51</v>
       </c>
     </row>
     <row r="84" spans="1:12" x14ac:dyDescent="0.25">
@@ -4228,7 +4228,7 @@
         <v>21</v>
       </c>
       <c r="L84">
-        <v>47</v>
+        <v>52</v>
       </c>
     </row>
     <row r="85" spans="1:12" x14ac:dyDescent="0.25">
@@ -4266,7 +4266,7 @@
         <v>21</v>
       </c>
       <c r="L85">
-        <v>47</v>
+        <v>52</v>
       </c>
     </row>
     <row r="86" spans="1:12" x14ac:dyDescent="0.25">
@@ -4304,7 +4304,7 @@
         <v>21</v>
       </c>
       <c r="L86">
-        <v>47</v>
+        <v>52</v>
       </c>
     </row>
     <row r="87" spans="1:12" x14ac:dyDescent="0.25">
@@ -4342,7 +4342,7 @@
         <v>21</v>
       </c>
       <c r="L87">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="88" spans="1:12" x14ac:dyDescent="0.25">
@@ -4380,7 +4380,7 @@
         <v>21</v>
       </c>
       <c r="L88">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="89" spans="1:12" x14ac:dyDescent="0.25">
@@ -4418,7 +4418,7 @@
         <v>21</v>
       </c>
       <c r="L89">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="90" spans="1:12" x14ac:dyDescent="0.25">
@@ -4456,7 +4456,7 @@
         <v>21</v>
       </c>
       <c r="L90">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="91" spans="1:12" x14ac:dyDescent="0.25">
@@ -4494,7 +4494,7 @@
         <v>21</v>
       </c>
       <c r="L91">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="92" spans="1:12" x14ac:dyDescent="0.25">
@@ -4532,7 +4532,7 @@
         <v>21</v>
       </c>
       <c r="L92">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="93" spans="1:12" x14ac:dyDescent="0.25">
@@ -4570,7 +4570,7 @@
         <v>21</v>
       </c>
       <c r="L93">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="94" spans="1:12" x14ac:dyDescent="0.25">
@@ -4608,7 +4608,7 @@
         <v>21</v>
       </c>
       <c r="L94">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="95" spans="1:12" x14ac:dyDescent="0.25">
@@ -4646,7 +4646,7 @@
         <v>21</v>
       </c>
       <c r="L95">
-        <v>51</v>
+        <v>56</v>
       </c>
     </row>
     <row r="96" spans="1:12" x14ac:dyDescent="0.25">
@@ -4684,7 +4684,7 @@
         <v>21</v>
       </c>
       <c r="L96">
-        <v>51</v>
+        <v>56</v>
       </c>
     </row>
     <row r="97" spans="1:12" x14ac:dyDescent="0.25">
@@ -4722,7 +4722,7 @@
         <v>21</v>
       </c>
       <c r="L97">
-        <v>51</v>
+        <v>56</v>
       </c>
     </row>
     <row r="98" spans="1:12" x14ac:dyDescent="0.25">
@@ -4760,7 +4760,7 @@
         <v>21</v>
       </c>
       <c r="L98">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="99" spans="1:12" x14ac:dyDescent="0.25">
@@ -4798,7 +4798,7 @@
         <v>21</v>
       </c>
       <c r="L99">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="100" spans="1:12" x14ac:dyDescent="0.25">
@@ -4836,7 +4836,7 @@
         <v>21</v>
       </c>
       <c r="L100">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="101" spans="1:12" x14ac:dyDescent="0.25">
@@ -4874,7 +4874,7 @@
         <v>21</v>
       </c>
       <c r="L101">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="102" spans="1:12" x14ac:dyDescent="0.25">
@@ -4912,7 +4912,7 @@
         <v>21</v>
       </c>
       <c r="L102">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="103" spans="1:12" x14ac:dyDescent="0.25">
@@ -4950,7 +4950,7 @@
         <v>21</v>
       </c>
       <c r="L103">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="104" spans="1:12" x14ac:dyDescent="0.25">
@@ -4988,7 +4988,7 @@
         <v>21</v>
       </c>
       <c r="L104">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="105" spans="1:12" x14ac:dyDescent="0.25">
@@ -5026,7 +5026,7 @@
         <v>21</v>
       </c>
       <c r="L105">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="106" spans="1:12" x14ac:dyDescent="0.25">
@@ -5064,7 +5064,7 @@
         <v>21</v>
       </c>
       <c r="L106">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="107" spans="1:12" x14ac:dyDescent="0.25">
@@ -5102,7 +5102,7 @@
         <v>21</v>
       </c>
       <c r="L107">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="108" spans="1:12" x14ac:dyDescent="0.25">
@@ -5140,7 +5140,7 @@
         <v>21</v>
       </c>
       <c r="L108">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="109" spans="1:12" x14ac:dyDescent="0.25">
@@ -5178,7 +5178,7 @@
         <v>21</v>
       </c>
       <c r="L109">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="110" spans="1:12" x14ac:dyDescent="0.25">
@@ -5216,7 +5216,7 @@
         <v>21</v>
       </c>
       <c r="L110">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="111" spans="1:12" x14ac:dyDescent="0.25">
@@ -5254,7 +5254,7 @@
         <v>21</v>
       </c>
       <c r="L111">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -5349,7 +5349,7 @@
         <v>206</v>
       </c>
       <c r="L2">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -5387,7 +5387,7 @@
         <v>206</v>
       </c>
       <c r="L3">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -5425,7 +5425,7 @@
         <v>206</v>
       </c>
       <c r="L4">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -5463,7 +5463,7 @@
         <v>206</v>
       </c>
       <c r="L5">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -5501,7 +5501,7 @@
         <v>206</v>
       </c>
       <c r="L6">
-        <v>32</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
@@ -5539,7 +5539,7 @@
         <v>206</v>
       </c>
       <c r="L7">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
@@ -5577,7 +5577,7 @@
         <v>206</v>
       </c>
       <c r="L8">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
@@ -5615,7 +5615,7 @@
         <v>206</v>
       </c>
       <c r="L9">
-        <v>46</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
@@ -5653,7 +5653,7 @@
         <v>206</v>
       </c>
       <c r="L10">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
@@ -5691,7 +5691,7 @@
         <v>206</v>
       </c>
       <c r="L11">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>